<commit_message>
audit: close D1a 0B-05C pre-execution checks
</commit_message>
<xml_diff>
--- a/docs/plan_fases_proyecto_investigacion_v0.1.xlsx
+++ b/docs/plan_fases_proyecto_investigacion_v0.1.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R41a6509bae2c4fca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementadas" sheetId="2" r:id="R2aff3dfdbf004f07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En_Ejecucion" sheetId="3" r:id="R52b2d316974d4c93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="4" r:id="R1a9d8529005a4a6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rb8e5f84010b9425b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementadas" sheetId="2" r:id="R7cdaf5f154d74cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En_Ejecucion" sheetId="3" r:id="R120696050fd14858"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="4" r:id="Rcfd358cd030a4c6f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -268,7 +268,7 @@
         <x:color rgb="FF065F46"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -279,7 +279,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -290,7 +290,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -301,7 +301,7 @@
         <x:color rgb="FF065F46"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -312,7 +312,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -323,7 +323,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -334,7 +334,7 @@
         <x:color rgb="FF065F46"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +345,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -356,7 +356,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -392,7 +392,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FasesActivas" displayName="FasesActivas" ref="A4:F7" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FasesActivas" displayName="FasesActivas" ref="A4:F8" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Fase"/>
     <x:tableColumn id="2" name="Estado"/>
@@ -462,9 +462,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -675,10 +675,10 @@
         <x:v>Fases en ejecución/preparación</x:v>
       </x:c>
       <x:c r="B6" s="26" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="26" t="str">
-        <x:v>LLM pre-retrieval, arquitectura visual y bibliografía local.</x:v>
+        <x:v>0B-05C D1a, LLM pre-retrieval, arquitectura visual y bibliografia local.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -697,10 +697,10 @@
         <x:v>Último estado técnico</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>Fase 5 cerrada</x:v>
+        <x:v>0B-05C cerrado prospectivamente</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>BM25 supera a Text2Trade dense; siguiente foco: LLM pre-retrieval con devset de 13 casos.</x:v>
+        <x:v>EXP-11B gate integrado; D1a sin exposicion de entrenamiento ni overlap Top-200. Sensibilidad numerica no autorizada.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -778,7 +778,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ab007b09ea476d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7648756bb140479f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -979,7 +979,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R120beda25e8b4382"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21c137536a5b4e79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1108,6 +1108,58 @@
         <x:v>Contar con referencias para pre-retrieval y model card/paper del LLM elegido.</x:v>
       </x:c>
     </x:row>
+    <x:row r="8" ht="195" hidden="0" customHeight="1">
+      <x:c r="A8" s="10" t="str">
+        <x:v>0B-05C - Auditoria pre-ejecucion D1a</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>Candidata para auditoria externa</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Resolver exposicion del optimizador y solapamiento Top-200; cerrar decisiones prospectivas.</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str">
+        <x:v>D1A_INDEX_EXPOSURE=CONFIRMED
+D1A_TRAINING_EXPOSURE=
+NO_EFFECTIVE_EXPOSURE_IDENTIFIED
+POSITIVE_EXPOSURE=NONE_IDENTIFIED
+EXPLICIT_HARD_NEGATIVE_EXPOSURE=
+NONE_IDENTIFIED
+IMPLICIT_IN_BATCH_EXPOSURE=
+NOT_IDENTIFIED
+D1A_RETRIEVAL_OUTPUT_OVERLAP=
+NONE_IDENTIFIED</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>MODEL_POLICY=
+FREEZE_ORIGINAL_D1A_WEIGHTS
+PRIMARY_CONTROL=
+FROZEN_ORIGINAL_D1A_OUTPUTS_FROM_
+DECISION_885_SNAPSHOT
+CORRECTED_INDEX_POLICY=
+FULL_ATOMIC_INDEX_AND_MAPPING_REBUILD
+OPTIONAL_CONTROL_REPRODUCTION=
+REPRODUCIBILITY_CHECK_ONLY
+D1A_EXECUTION_SPECIFICATION=
+CLOSED_PROSPECTIVELY
+D1A_METRIC_IMPACT=NOT_DETERMINED</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="str">
+        <x:v>D1A_NUMERICAL_EXECUTION=
+NOT_AUTHORIZED
+DOWNSTREAM_REEXECUTION=
+NOT_YET_JUSTIFIED
+0B05C_CLOSURE=NOT_AUTHORIZED
+EXP11B_RETRIEVAL_GATE=
+APPROVED_AND_INTEGRATED
+EXP11B_RETRIEVAL_EXECUTION=
+NOT_AUTHORIZED
+RETRIEVAL_EXECUTED=false
+EVALUATION_METRICS_COMPUTED=false
+H150_H200_RESULTS_OBSERVED=false
+EXP12_AUTHORIZED=false</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -1120,7 +1172,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01ec28c8690d4b9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdb4e1dc890d411e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1341,7 +1393,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bbf463f6a304d2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a6464f8b18140d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: close D1a 0B-05C evidence microclose
</commit_message>
<xml_diff>
--- a/docs/plan_fases_proyecto_investigacion_v0.1.xlsx
+++ b/docs/plan_fases_proyecto_investigacion_v0.1.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rb8e5f84010b9425b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementadas" sheetId="2" r:id="R7cdaf5f154d74cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En_Ejecucion" sheetId="3" r:id="R120696050fd14858"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="4" r:id="Rcfd358cd030a4c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R41a6509bae2c4fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementadas" sheetId="2" r:id="R2aff3dfdbf004f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En_Ejecucion" sheetId="3" r:id="R52b2d316974d4c93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="4" r:id="R1a9d8529005a4a6f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -268,7 +268,7 @@
         <x:color rgb="FF065F46"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -279,7 +279,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -290,7 +290,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -301,7 +301,7 @@
         <x:color rgb="FF065F46"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -312,7 +312,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -323,7 +323,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -334,7 +334,7 @@
         <x:color rgb="FF065F46"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +345,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -356,7 +356,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -392,7 +392,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FasesActivas" displayName="FasesActivas" ref="A4:F8" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FasesActivas" displayName="FasesActivas" ref="A4:F7" headerRowCount="1">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Fase"/>
     <x:tableColumn id="2" name="Estado"/>
@@ -462,9 +462,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Calibri Light"/>
-        <a:cs typeface="Calibri Light"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -675,10 +675,10 @@
         <x:v>Fases en ejecución/preparación</x:v>
       </x:c>
       <x:c r="B6" s="26" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="26" t="str">
-        <x:v>0B-05C D1a, LLM pre-retrieval, arquitectura visual y bibliografia local.</x:v>
+        <x:v>LLM pre-retrieval, arquitectura visual y bibliografía local.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -697,10 +697,10 @@
         <x:v>Último estado técnico</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>0B-05C cerrado prospectivamente</x:v>
+        <x:v>Fase 5 cerrada</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>EXP-11B gate integrado; D1a sin exposicion de entrenamiento ni overlap Top-200. Sensibilidad numerica no autorizada.</x:v>
+        <x:v>BM25 supera a Text2Trade dense; siguiente foco: LLM pre-retrieval con devset de 13 casos.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -778,7 +778,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7648756bb140479f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ab007b09ea476d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -979,7 +979,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21c137536a5b4e79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R120beda25e8b4382"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1108,58 +1108,6 @@
         <x:v>Contar con referencias para pre-retrieval y model card/paper del LLM elegido.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="195" hidden="0" customHeight="1">
-      <x:c r="A8" s="10" t="str">
-        <x:v>0B-05C - Auditoria pre-ejecucion D1a</x:v>
-      </x:c>
-      <x:c r="B8" s="10" t="str">
-        <x:v>Candidata para auditoria externa</x:v>
-      </x:c>
-      <x:c r="C8" s="10" t="str">
-        <x:v>Resolver exposicion del optimizador y solapamiento Top-200; cerrar decisiones prospectivas.</x:v>
-      </x:c>
-      <x:c r="D8" s="10" t="str">
-        <x:v>D1A_INDEX_EXPOSURE=CONFIRMED
-D1A_TRAINING_EXPOSURE=
-NO_EFFECTIVE_EXPOSURE_IDENTIFIED
-POSITIVE_EXPOSURE=NONE_IDENTIFIED
-EXPLICIT_HARD_NEGATIVE_EXPOSURE=
-NONE_IDENTIFIED
-IMPLICIT_IN_BATCH_EXPOSURE=
-NOT_IDENTIFIED
-D1A_RETRIEVAL_OUTPUT_OVERLAP=
-NONE_IDENTIFIED</x:v>
-      </x:c>
-      <x:c r="E8" s="10" t="str">
-        <x:v>MODEL_POLICY=
-FREEZE_ORIGINAL_D1A_WEIGHTS
-PRIMARY_CONTROL=
-FROZEN_ORIGINAL_D1A_OUTPUTS_FROM_
-DECISION_885_SNAPSHOT
-CORRECTED_INDEX_POLICY=
-FULL_ATOMIC_INDEX_AND_MAPPING_REBUILD
-OPTIONAL_CONTROL_REPRODUCTION=
-REPRODUCIBILITY_CHECK_ONLY
-D1A_EXECUTION_SPECIFICATION=
-CLOSED_PROSPECTIVELY
-D1A_METRIC_IMPACT=NOT_DETERMINED</x:v>
-      </x:c>
-      <x:c r="F8" s="10" t="str">
-        <x:v>D1A_NUMERICAL_EXECUTION=
-NOT_AUTHORIZED
-DOWNSTREAM_REEXECUTION=
-NOT_YET_JUSTIFIED
-0B05C_CLOSURE=NOT_AUTHORIZED
-EXP11B_RETRIEVAL_GATE=
-APPROVED_AND_INTEGRATED
-EXP11B_RETRIEVAL_EXECUTION=
-NOT_AUTHORIZED
-RETRIEVAL_EXECUTED=false
-EVALUATION_METRICS_COMPUTED=false
-H150_H200_RESULTS_OBSERVED=false
-EXP12_AUTHORIZED=false</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -1172,7 +1120,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdb4e1dc890d411e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01ec28c8690d4b9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1393,7 +1341,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a6464f8b18140d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bbf463f6a304d2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>